<commit_message>
Finalize QA testing portfolio project
</commit_message>
<xml_diff>
--- a/04-Bug-Reports/Bug-Reports.xlsx
+++ b/04-Bug-Reports/Bug-Reports.xlsx
@@ -7,9 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bug Reports" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Defect Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Failed Test Investigation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Blocked Test Investigation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Defect Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Log'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Failed Test Investigation'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Blocked Test Investigation'!$A$1:$F$19</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,12 +37,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
-    <font>
-      <i val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -44,8 +47,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED7D31"/>
+        <bgColor rgb="00ED7D31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+        <bgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,15 +88,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,22 +470,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,88 +495,1195 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Severity</t>
+          <t>Steps to Reproduce</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Reproducibility</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Evidence Screenshot</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Linked Test Case</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>No bugs to report — tests were not executed due to absence of Android execution environment</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>All 37 executed test cases</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>No confirmed application defects identified</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>All Modules</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pixel 8 Emulator, Android 17, API 37</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>All 37 test cases were executed against a real Android emulator. 5 FAIL and 18 BLOCKED results were investigated.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Application functions as designed</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>No genuine application defects found. All failures/blockers were caused by test automation UI element location limitations, not application defects.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED - NO DEFECT</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:M2"/>
-  </mergeCells>
+  <autoFilter ref="A1:L2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Screenshot</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed Defect ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Verify app launch / home screen display</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Catalog not visible</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not verify catalog display on app launch. The app launched but the automated script's UI element detection for the catalog grid failed.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-001.png</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Menu accessibility</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Menu did not open</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script attempted to open the navigation menu but could not locate/trigger the menu button via UIAutomator.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-002.png</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-009</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Product catalog display</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Product list not visible</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not detect the product list elements on the catalog screen.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-009.png</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-014</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Product details view</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Product detail view not displayed correctly</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not verify the product detail view layout due to UI element detection limitations.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-014.png</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>App relaunch to catalog</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>App did not relaunch to catalog</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not verify the app relaunch behavior returned to the catalog screen.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-036.png</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Reason Blocked</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Evidence Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-004</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Login screen navigation</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Log In not found in menu</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the "Log In" menu item via UIAutomator.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-005</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Invalid login handling</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Could not navigate to login screen.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not navigate to the login screen because the login menu item was not locatable.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-006</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Empty login fields</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Not on login screen.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not verify it was on the login screen.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-007</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Login success navigation</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Not on login screen.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not verify it was on the login screen.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-010</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Product listing with details</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sort options not found</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate sort options on the catalog screen.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-011</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Product sorting - A to Z</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Z-A sort option not found</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the Z-A sort option.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-011.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-012</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Product sorting - price low to high</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Price ascending sort not found</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the price ascending sort option.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-012.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-013</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Product sorting - price high to low</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Price descending sort not found</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the price descending sort option.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Add to cart button (product detail)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Plus button not found on product detail.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the plus (+) button on the product detail screen.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-016.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Increase quantity (product detail)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Minus button not found on product detail.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the minus (-) button on the product detail screen.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-017.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease quantity (product detail)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Cannot test - minus button not found.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the minus (-) button, preventing quantity decrease testing.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-018.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Add to cart functionality</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Add To Cart button not found.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the "Add To Cart" button.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-019.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Cart items visibility</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Cart may be empty or items not visible.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not verify cart items were visible.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-021.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Increase cart quantity</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Plus button not found in cart.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the plus (+) button in the cart view.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-022.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Decrease cart quantity</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Minus button not found in cart.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the minus (-) button in the cart view.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-023.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Remove item from cart</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Remove button not found in cart.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the remove button in the cart view.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-024.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>QR code scanner feature</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>QR Code Scanner not found in menu.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the QR Code Scanner menu item.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-035.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Add to cart (repeated test)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Add To Cart not found for repeated test.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Test automation script could not locate the "Add To Cart" button during the repeated test.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issue</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>07-Screenshots/application/TC-037.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Total Tests Executed</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Total Tests Investigated</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Failed Tests Investigated</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Blocked Tests Investigated</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed Application Defects</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Automation/Locator Issues</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Environment Issues</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Test Data Issues</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Not Reproducible</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Pass Rate</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>35.1% (13/37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Critical Path Pass Rate</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>100% (9/9 checkout flow)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>